<commit_message>
Chamol PO: remove comment heading and quote reference
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoEh7Mj6ZxttHm1PyDH2Zo
</commit_message>
<xml_diff>
--- a/outputs/PO_Woodlite_Chamol.xlsx
+++ b/outputs/PO_Woodlite_Chamol.xlsx
@@ -4835,7 +4835,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{385F0503-BD0D-401C-8C6C-42B65B8A1060}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{924A07AF-7E5A-4B88-9BCA-E6B846CBC9A5}">
   <dimension ref="A2:G106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5132,17 +5132,11 @@
       <c r="A28" s="6"/>
     </row>
     <row r="29" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="99" t="s">
-        <v>17</v>
-      </c>
+      <c r="A29" s="99"/>
       <c r="B29" s="88"/>
     </row>
     <row r="30" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ref: Chamol Quote No. QN261012F018</t>
-        </is>
-      </c>
+      <c r="A30" s="69"/>
       <c r="B30" s="74"/>
     </row>
     <row r="31" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5395,8 +5389,8 @@
     <mergeCell ref="A45:B45"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{E243124E-42BE-43E6-9CEF-D3D5C9C378A5}"/>
-    <hyperlink ref="A40" r:id="rId2" xr:uid="{FFB5AB89-7FD8-4DFC-A859-EAC87EE87FB5}"/>
+    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{6E951400-B871-4EE0-A5FD-45B86C6A8B66}"/>
+    <hyperlink ref="A40" r:id="rId2" xr:uid="{8EE7B13A-B00E-4B61-B20D-30967937CA8F}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="1.1299999999999999" bottom="0.75" header="0.35" footer="0.3"/>
   <pageSetup scale="78" orientation="portrait" r:id="rId3"/>

</xml_diff>

<commit_message>
Chamol PO: remove the comment/payment box from page 1
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoEh7Mj6ZxttHm1PyDH2Zo
</commit_message>
<xml_diff>
--- a/outputs/PO_Woodlite_Chamol.xlsx
+++ b/outputs/PO_Woodlite_Chamol.xlsx
@@ -4835,7 +4835,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{924A07AF-7E5A-4B88-9BCA-E6B846CBC9A5}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3082F410-5E78-4070-81DC-D803373CD69D}">
   <dimension ref="A2:G106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -5131,19 +5131,9 @@
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
     </row>
-    <row r="29" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="99"/>
-      <c r="B29" s="88"/>
-    </row>
-    <row r="30" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="69"/>
-      <c r="B30" s="74"/>
-    </row>
+    <row r="29" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="31" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="109" t="s">
-        <v>19</v>
-      </c>
-      <c r="B31" s="110"/>
       <c r="C31" s="6"/>
       <c r="E31" s="17" t="s">
         <v>22</v>
@@ -5151,96 +5141,54 @@
       <c r="F31" s="10"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" s="69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1) 50% Advance, balance before shipment by T/T</t>
-        </is>
-      </c>
-      <c r="B32" s="70"/>
       <c r="C32" s="6"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2) Excluding V.A.T</t>
-        </is>
-      </c>
-      <c r="B33" s="70"/>
       <c r="C33" s="6"/>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" s="69" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3) Delivery: 30 days after advance payment</t>
-        </is>
-      </c>
-      <c r="B34" s="113"/>
       <c r="C34" s="6"/>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" s="69" t="s">
-        <v>27</v>
-      </c>
-      <c r="B35" s="70"/>
       <c r="C35" s="6"/>
       <c r="D35" s="10"/>
       <c r="E35" s="16"/>
       <c r="F35" s="16"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" s="69" t="s">
-        <v>23</v>
-      </c>
-      <c r="B36" s="70"/>
       <c r="C36" s="6"/>
       <c r="D36" s="10"/>
       <c r="E36" s="16"/>
       <c r="F36" s="16"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" s="69" t="s">
-        <v>24</v>
-      </c>
-      <c r="B37" s="70"/>
       <c r="C37" s="6"/>
       <c r="D37" s="10"/>
       <c r="E37" s="16"/>
       <c r="F37" s="16"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="69" t="s">
-        <v>25</v>
-      </c>
-      <c r="B38" s="70"/>
       <c r="C38" s="6"/>
       <c r="D38" s="10"/>
       <c r="E38" s="16"/>
       <c r="F38" s="16"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" s="71" t="s">
-        <v>26</v>
-      </c>
-      <c r="B39" s="72"/>
       <c r="C39" s="6"/>
       <c r="D39" s="10"/>
       <c r="E39" s="16"/>
       <c r="F39" s="16"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" s="89" t="s">
-        <v>10</v>
-      </c>
-      <c r="B40" s="111"/>
       <c r="C40" s="6"/>
       <c r="D40" s="10"/>
       <c r="E40" s="16"/>
@@ -5389,8 +5337,8 @@
     <mergeCell ref="A45:B45"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{6E951400-B871-4EE0-A5FD-45B86C6A8B66}"/>
-    <hyperlink ref="A40" r:id="rId2" xr:uid="{8EE7B13A-B00E-4B61-B20D-30967937CA8F}"/>
+    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{7862171A-2B6B-410E-AC22-F6F4FDFC6D01}"/>
+    <hyperlink ref="A40" r:id="rId2" xr:uid="{60CCF669-9ADA-438F-A133-EF7517669274}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="1.1299999999999999" bottom="0.75" header="0.35" footer="0.3"/>
   <pageSetup scale="78" orientation="portrait" r:id="rId3"/>

</xml_diff>

<commit_message>
Chamol PO: show full PURCHASE ORDER title, close gap, tidy item description
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoEh7Mj6ZxttHm1PyDH2Zo
</commit_message>
<xml_diff>
--- a/outputs/PO_Woodlite_Chamol.xlsx
+++ b/outputs/PO_Woodlite_Chamol.xlsx
@@ -784,7 +784,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="153">
+  <cellXfs count="154">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1143,6 +1143,9 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -4835,7 +4838,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3082F410-5E78-4070-81DC-D803373CD69D}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC9DF5E0-3A7D-40E9-8AF8-2DB75BF48A39}">
   <dimension ref="A2:G106"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -4849,9 +4852,11 @@
   <sheetData>
     <row r="2" spans="1:7" ht="35.25" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A2" s="1"/>
-      <c r="E2" s="42" t="s">
+      <c r="D2" s="153" t="s">
         <v>15</v>
       </c>
+      <c r="E2" s="153"/>
+      <c r="F2" s="153"/>
     </row>
     <row r="3" spans="1:7" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E3" s="43" t="s">
@@ -5064,7 +5069,8 @@
       </c>
       <c r="B23" s="129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spiral Bevel Gear Set (18CrNiMo7-6)</t>
+          <t xml:space="preserve">Spiral Bevel Gear Set
+(18CrNiMo7-6)</t>
         </is>
       </c>
       <c r="C23" s="129">
@@ -5131,64 +5137,64 @@
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
     </row>
-    <row r="29" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" hidden="1" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" hidden="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" hidden="1" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C31" s="6"/>
       <c r="E31" s="17" t="s">
         <v>22</v>
       </c>
       <c r="F31" s="10"/>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" hidden="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C32" s="6"/>
       <c r="D32" s="10"/>
       <c r="E32" s="10"/>
       <c r="F32" s="10"/>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="33" hidden="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C33" s="6"/>
       <c r="D33" s="10"/>
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="34" hidden="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C34" s="6"/>
       <c r="D34" s="10"/>
       <c r="E34" s="10"/>
       <c r="F34" s="10"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="35" hidden="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C35" s="6"/>
       <c r="D35" s="10"/>
       <c r="E35" s="16"/>
       <c r="F35" s="16"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="36" hidden="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C36" s="6"/>
       <c r="D36" s="10"/>
       <c r="E36" s="16"/>
       <c r="F36" s="16"/>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="37" hidden="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C37" s="6"/>
       <c r="D37" s="10"/>
       <c r="E37" s="16"/>
       <c r="F37" s="16"/>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="38" hidden="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C38" s="6"/>
       <c r="D38" s="10"/>
       <c r="E38" s="16"/>
       <c r="F38" s="16"/>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="39" hidden="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C39" s="6"/>
       <c r="D39" s="10"/>
       <c r="E39" s="16"/>
       <c r="F39" s="16"/>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="40" hidden="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C40" s="6"/>
       <c r="D40" s="10"/>
       <c r="E40" s="16"/>
@@ -5292,7 +5298,8 @@
       <c r="F52" s="37"/>
     </row>
   </sheetData>
-  <mergeCells count="42">
+  <mergeCells count="43">
+    <mergeCell ref="D2:F2"/>
     <mergeCell ref="F25:F26"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="E9:F9"/>
@@ -5337,8 +5344,7 @@
     <mergeCell ref="A45:B45"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{7862171A-2B6B-410E-AC22-F6F4FDFC6D01}"/>
-    <hyperlink ref="A40" r:id="rId2" xr:uid="{60CCF669-9ADA-438F-A133-EF7517669274}"/>
+    <hyperlink ref="A15" r:id="rId1" display="mailto:woodlite18@gmail.com" xr:uid="{9BB12F07-61EA-46FC-A013-BA88637D9232}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="1.1299999999999999" bottom="0.75" header="0.35" footer="0.3"/>
   <pageSetup scale="78" orientation="portrait" r:id="rId3"/>

</xml_diff>